<commit_message>
Update Land Policy FOPITY
</commit_message>
<xml_diff>
--- a/InputData/land/CSpULApYbP/na-CO2 Sequestered per Unit Land Area per Year by Pol.xlsx
+++ b/InputData/land/CSpULApYbP/na-CO2 Sequestered per Unit Land Area per Year by Pol.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\EPS\Github Push\China\eps-china2019-smart-trans\InputData\land\CSpULApYbP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Land\CSpULApYbP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DFB1CE-8AF0-4739-84B2-83EBB98A4446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC6AB99-C3D9-4ECE-A72B-B31E8B3AE152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23925" yWindow="2070" windowWidth="21600" windowHeight="11385" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
   <externalReferences>
     <externalReference r:id="rId5"/>
     <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <definedNames>
     <definedName name="acres_per_hectare">#REF!</definedName>
@@ -948,6 +949,39 @@
 </externalLink>
 </file>
 
+<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+      <sheetName val="About"/>
+      <sheetName val="Calculations"/>
+      <sheetName val="na-CO2 Abated per Unit Land Are"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="9">
+          <cell r="J9">
+            <v>250883.0340962171</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="J15">
+            <v>81612.28743035956</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -2659,7 +2693,8 @@
         <v>4</v>
       </c>
       <c r="B3" s="3">
-        <v>91741.808767074341</v>
+        <f>[3]Sheet1!$J$15</f>
+        <v>81612.28743035956</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -2793,7 +2828,8 @@
         <v>8</v>
       </c>
       <c r="B7" s="3">
-        <v>194930.20678155916</v>
+        <f>[3]Sheet1!$J$9</f>
+        <v>250883.0340962171</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -2837,6 +2873,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="文档" ma:contentTypeID="0x010100BD1DE36A36CC7845A4126EF01914151E" ma:contentTypeVersion="14" ma:contentTypeDescription="新建文档。" ma:contentTypeScope="" ma:versionID="310835f059701aa681930bc3a1715053">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="2e2398b5-f60e-4ca0-a4ba-6048b5e4e90c" xmlns:ns3="a06c533b-533a-4f75-b7db-110f073002e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7ba933288dd05553e9ce0f804d4dc608" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3070,7 +3115,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3079,16 +3124,17 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2887E70D-36D4-4813-B132-0547119682E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4A54D4F-A403-4885-89C5-492780163B87}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3108,20 +3154,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0ADDB5C7-ECC4-4C51-99FE-CBD4F31EF89A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2887E70D-36D4-4813-B132-0547119682E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>